<commit_message>
docs: point Excel evidence links to Word documents and remove intro headers
</commit_message>
<xml_diff>
--- a/docs/Report/SWP_SE20A05_Group7_ReportAI.xlsx
+++ b/docs/Report/SWP_SE20A05_Group7_ReportAI.xlsx
@@ -1927,7 +1927,7 @@
       </c>
       <c r="G2" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week9.md#task-1-campaign-completion-pipeline</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week9.docx</t>
         </is>
       </c>
       <c r="H2" s="30" t="inlineStr">
@@ -1977,7 +1977,7 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week9.md#task-2-gemini-key-rotation</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week9.docx</t>
         </is>
       </c>
       <c r="H3" s="30" t="inlineStr">
@@ -2027,7 +2027,7 @@
       </c>
       <c r="G4" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week9.md#task-3-google-oauth-session-preservation</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week9.docx</t>
         </is>
       </c>
       <c r="H4" s="30" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="G5" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week9.md#task-4-recruitment-request-ui-alignment</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week9.docx</t>
         </is>
       </c>
       <c r="H5" s="30" t="inlineStr">
@@ -2311,7 +2311,7 @@
       </c>
       <c r="G2" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week10.md#task-1-playwright-e2e-testing</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week10.docx</t>
         </is>
       </c>
       <c r="H2" s="30" t="inlineStr">
@@ -2361,7 +2361,7 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week10.md#task-2-postman-newman-runner</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week10.docx</t>
         </is>
       </c>
       <c r="H3" s="30" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="G4" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week10.md#task-3-issues-report-sync-automation</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week10.docx</t>
         </is>
       </c>
       <c r="H4" s="30" t="inlineStr">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="G2" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week1.md#task-1-candidate-search-strategy</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week1.docx</t>
         </is>
       </c>
       <c r="H2" s="30" t="inlineStr">
@@ -2732,7 +2732,7 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week1.md#task-2-database-schema-erd-design</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week1.docx</t>
         </is>
       </c>
       <c r="H3" s="30" t="inlineStr">
@@ -3890,7 +3890,7 @@
       </c>
       <c r="G2" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week2.md#task-1-global-jwtauthguard-in-gateway</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week2.docx</t>
         </is>
       </c>
       <c r="H2" s="30" t="inlineStr">
@@ -3954,7 +3954,7 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week2.md#task-2-jest-integration-testing-for-unauthorized-requests</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week2.docx</t>
         </is>
       </c>
       <c r="H3" s="30" t="inlineStr">
@@ -4018,7 +4018,7 @@
       </c>
       <c r="G4" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week2.md#task-3-public-endpoint-controller-testing</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week2.docx</t>
         </is>
       </c>
       <c r="H4" s="30" t="inlineStr">
@@ -4082,7 +4082,7 @@
       </c>
       <c r="G5" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week2.md#task-4-logout-token-invalidation-strategy</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week2.docx</t>
         </is>
       </c>
       <c r="H5" s="30" t="inlineStr">
@@ -4146,7 +4146,7 @@
       </c>
       <c r="G6" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week2.md#task-5-redis-logout-keyspace-design</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week2.docx</t>
         </is>
       </c>
       <c r="H6" s="30" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="G7" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week2.md#task-6-post-logout-refresh-testing</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week2.docx</t>
         </is>
       </c>
       <c r="H7" s="30" t="inlineStr">
@@ -4274,7 +4274,7 @@
       </c>
       <c r="G8" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week2.md#task-7-jwt-header-extraction</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week2.docx</t>
         </is>
       </c>
       <c r="H8" s="30" t="inlineStr">
@@ -32276,7 +32276,7 @@
       </c>
       <c r="G2" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week3.md#task-1-organizationservice-crud</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week3.docx</t>
         </is>
       </c>
       <c r="H2" s="30" t="inlineStr">
@@ -32326,7 +32326,7 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week3.md#task-2-departmentservice-unit-tests</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week3.docx</t>
         </is>
       </c>
       <c r="H3" s="30" t="inlineStr">
@@ -32376,7 +32376,7 @@
       </c>
       <c r="G4" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week3.md#task-3-approvalchain-sequential-level-testing</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week3.docx</t>
         </is>
       </c>
       <c r="H4" s="30" t="inlineStr">
@@ -32426,7 +32426,7 @@
       </c>
       <c r="G5" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week3.md#task-4-prisma-transaction-mocking</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week3.docx</t>
         </is>
       </c>
       <c r="H5" s="30" t="inlineStr">
@@ -32649,7 +32649,7 @@
       </c>
       <c r="G2" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week4.md#task-1-multi-tenant-rolesguard</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week4.docx</t>
         </is>
       </c>
       <c r="H2" s="30" t="inlineStr">
@@ -32699,7 +32699,7 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week4.md#task-2-user-context-propagation-via-tcp</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week4.docx</t>
         </is>
       </c>
       <c r="H3" s="30" t="inlineStr">
@@ -32749,7 +32749,7 @@
       </c>
       <c r="G4" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week4.md#task-3-multi-tenant-isolation-tests</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week4.docx</t>
         </is>
       </c>
       <c r="H4" s="30" t="inlineStr">
@@ -32986,7 +32986,7 @@
       </c>
       <c r="G2" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week5.md#task-1-approval-request-sequential-transitions</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week5.docx</t>
         </is>
       </c>
       <c r="H2" s="30" t="inlineStr">
@@ -33036,7 +33036,7 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week5.md#task-2-bullmq-async-notifications-queue</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week5.docx</t>
         </is>
       </c>
       <c r="H3" s="30" t="inlineStr">
@@ -33086,7 +33086,7 @@
       </c>
       <c r="G4" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week5.md#task-3-approval-concurrency-testing</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week5.docx</t>
         </is>
       </c>
       <c r="H4" s="30" t="inlineStr">
@@ -33323,7 +33323,7 @@
       </c>
       <c r="G2" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week6.md#task-1-microservice-exception-filters</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week6.docx</t>
         </is>
       </c>
       <c r="H2" s="30" t="inlineStr">
@@ -33373,7 +33373,7 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week6.md#task-2-redis-cache-strategy</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week6.docx</t>
         </is>
       </c>
       <c r="H3" s="30" t="inlineStr">
@@ -33423,7 +33423,7 @@
       </c>
       <c r="G4" s="33" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week6.md#task-3-resolving-prisma-n1-issues</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week6.docx</t>
         </is>
       </c>
       <c r="H4" s="30" t="inlineStr">
@@ -33473,7 +33473,7 @@
       </c>
       <c r="G5" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week6.md#task-4-vector-search-ai-model-evaluation</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week6.docx</t>
         </is>
       </c>
       <c r="H5" s="30" t="inlineStr">
@@ -33696,7 +33696,7 @@
       </c>
       <c r="G2" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week7.md#task-1-cv-file-parser-pipeline</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week7.docx</t>
         </is>
       </c>
       <c r="H2" s="30" t="inlineStr">
@@ -33746,7 +33746,7 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week7.md#task-2-candidate-portal-api</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week7.docx</t>
         </is>
       </c>
       <c r="H3" s="30" t="inlineStr">
@@ -33796,7 +33796,7 @@
       </c>
       <c r="G4" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week7.md#task-3-cv-replacement-transaction</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week7.docx</t>
         </is>
       </c>
       <c r="H4" s="30" t="inlineStr">
@@ -33846,7 +33846,7 @@
       </c>
       <c r="G5" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week7.md#task-4-hybrid-candidate-search</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week7.docx</t>
         </is>
       </c>
       <c r="H5" s="30" t="inlineStr">
@@ -33896,7 +33896,7 @@
       </c>
       <c r="G6" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week7.md#task-5-interview-feedback-permissions</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week7.docx</t>
         </is>
       </c>
       <c r="H6" s="30" t="inlineStr">
@@ -34116,7 +34116,7 @@
       </c>
       <c r="G2" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week8.md#task-1-evaluation-scores-refinement</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week8.docx</t>
         </is>
       </c>
       <c r="H2" s="30" t="inlineStr">
@@ -34166,7 +34166,7 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week8.md#task-2-gateway-routes-verification</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week8.docx</t>
         </is>
       </c>
       <c r="H3" s="30" t="inlineStr">
@@ -34216,7 +34216,7 @@
       </c>
       <c r="G4" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week8.md#task-3-screen-flows-plantuml</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week8.docx</t>
         </is>
       </c>
       <c r="H4" s="30" t="inlineStr">
@@ -34266,7 +34266,7 @@
       </c>
       <c r="G5" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week8.md#task-4-traceability-matrix</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week8.docx</t>
         </is>
       </c>
       <c r="H5" s="30" t="inlineStr">
@@ -34316,7 +34316,7 @@
       </c>
       <c r="G6" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week8.md#task-5-project-reports-compilation</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week8.docx</t>
         </is>
       </c>
       <c r="H6" s="30" t="inlineStr">

</xml_diff>

<commit_message>
docs: use correct branch name in Excel evidence links
</commit_message>
<xml_diff>
--- a/docs/Report/SWP_SE20A05_Group7_ReportAI.xlsx
+++ b/docs/Report/SWP_SE20A05_Group7_ReportAI.xlsx
@@ -1927,7 +1927,7 @@
       </c>
       <c r="G2" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week9.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week9.docx</t>
         </is>
       </c>
       <c r="H2" s="30" t="inlineStr">
@@ -1977,7 +1977,7 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week9.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week9.docx</t>
         </is>
       </c>
       <c r="H3" s="30" t="inlineStr">
@@ -2027,7 +2027,7 @@
       </c>
       <c r="G4" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week9.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week9.docx</t>
         </is>
       </c>
       <c r="H4" s="30" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="G5" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week9.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week9.docx</t>
         </is>
       </c>
       <c r="H5" s="30" t="inlineStr">
@@ -2311,7 +2311,7 @@
       </c>
       <c r="G2" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week10.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week10.docx</t>
         </is>
       </c>
       <c r="H2" s="30" t="inlineStr">
@@ -2361,7 +2361,7 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week10.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week10.docx</t>
         </is>
       </c>
       <c r="H3" s="30" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="G4" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week10.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week10.docx</t>
         </is>
       </c>
       <c r="H4" s="30" t="inlineStr">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="G2" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week1.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week1.docx</t>
         </is>
       </c>
       <c r="H2" s="30" t="inlineStr">
@@ -2732,7 +2732,7 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week1.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week1.docx</t>
         </is>
       </c>
       <c r="H3" s="30" t="inlineStr">
@@ -3890,7 +3890,7 @@
       </c>
       <c r="G2" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week2.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week2.docx</t>
         </is>
       </c>
       <c r="H2" s="30" t="inlineStr">
@@ -3954,7 +3954,7 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week2.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week2.docx</t>
         </is>
       </c>
       <c r="H3" s="30" t="inlineStr">
@@ -4018,7 +4018,7 @@
       </c>
       <c r="G4" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week2.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week2.docx</t>
         </is>
       </c>
       <c r="H4" s="30" t="inlineStr">
@@ -4082,7 +4082,7 @@
       </c>
       <c r="G5" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week2.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week2.docx</t>
         </is>
       </c>
       <c r="H5" s="30" t="inlineStr">
@@ -4146,7 +4146,7 @@
       </c>
       <c r="G6" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week2.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week2.docx</t>
         </is>
       </c>
       <c r="H6" s="30" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="G7" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week2.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week2.docx</t>
         </is>
       </c>
       <c r="H7" s="30" t="inlineStr">
@@ -4274,7 +4274,7 @@
       </c>
       <c r="G8" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week2.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week2.docx</t>
         </is>
       </c>
       <c r="H8" s="30" t="inlineStr">
@@ -32276,7 +32276,7 @@
       </c>
       <c r="G2" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week3.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week3.docx</t>
         </is>
       </c>
       <c r="H2" s="30" t="inlineStr">
@@ -32326,7 +32326,7 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week3.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week3.docx</t>
         </is>
       </c>
       <c r="H3" s="30" t="inlineStr">
@@ -32376,7 +32376,7 @@
       </c>
       <c r="G4" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week3.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week3.docx</t>
         </is>
       </c>
       <c r="H4" s="30" t="inlineStr">
@@ -32426,7 +32426,7 @@
       </c>
       <c r="G5" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week3.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week3.docx</t>
         </is>
       </c>
       <c r="H5" s="30" t="inlineStr">
@@ -32649,7 +32649,7 @@
       </c>
       <c r="G2" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week4.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week4.docx</t>
         </is>
       </c>
       <c r="H2" s="30" t="inlineStr">
@@ -32699,7 +32699,7 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week4.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week4.docx</t>
         </is>
       </c>
       <c r="H3" s="30" t="inlineStr">
@@ -32749,7 +32749,7 @@
       </c>
       <c r="G4" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week4.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week4.docx</t>
         </is>
       </c>
       <c r="H4" s="30" t="inlineStr">
@@ -32986,7 +32986,7 @@
       </c>
       <c r="G2" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week5.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week5.docx</t>
         </is>
       </c>
       <c r="H2" s="30" t="inlineStr">
@@ -33036,7 +33036,7 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week5.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week5.docx</t>
         </is>
       </c>
       <c r="H3" s="30" t="inlineStr">
@@ -33086,7 +33086,7 @@
       </c>
       <c r="G4" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week5.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week5.docx</t>
         </is>
       </c>
       <c r="H4" s="30" t="inlineStr">
@@ -33323,7 +33323,7 @@
       </c>
       <c r="G2" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week6.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week6.docx</t>
         </is>
       </c>
       <c r="H2" s="30" t="inlineStr">
@@ -33373,7 +33373,7 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week6.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week6.docx</t>
         </is>
       </c>
       <c r="H3" s="30" t="inlineStr">
@@ -33423,7 +33423,7 @@
       </c>
       <c r="G4" s="33" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week6.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week6.docx</t>
         </is>
       </c>
       <c r="H4" s="30" t="inlineStr">
@@ -33473,7 +33473,7 @@
       </c>
       <c r="G5" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week6.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week6.docx</t>
         </is>
       </c>
       <c r="H5" s="30" t="inlineStr">
@@ -33696,7 +33696,7 @@
       </c>
       <c r="G2" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week7.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week7.docx</t>
         </is>
       </c>
       <c r="H2" s="30" t="inlineStr">
@@ -33746,7 +33746,7 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week7.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week7.docx</t>
         </is>
       </c>
       <c r="H3" s="30" t="inlineStr">
@@ -33796,7 +33796,7 @@
       </c>
       <c r="G4" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week7.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week7.docx</t>
         </is>
       </c>
       <c r="H4" s="30" t="inlineStr">
@@ -33846,7 +33846,7 @@
       </c>
       <c r="G5" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week7.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week7.docx</t>
         </is>
       </c>
       <c r="H5" s="30" t="inlineStr">
@@ -33896,7 +33896,7 @@
       </c>
       <c r="G6" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week7.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week7.docx</t>
         </is>
       </c>
       <c r="H6" s="30" t="inlineStr">
@@ -34116,7 +34116,7 @@
       </c>
       <c r="G2" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week8.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week8.docx</t>
         </is>
       </c>
       <c r="H2" s="30" t="inlineStr">
@@ -34166,7 +34166,7 @@
       </c>
       <c r="G3" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week8.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week8.docx</t>
         </is>
       </c>
       <c r="H3" s="30" t="inlineStr">
@@ -34216,7 +34216,7 @@
       </c>
       <c r="G4" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week8.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week8.docx</t>
         </is>
       </c>
       <c r="H4" s="30" t="inlineStr">
@@ -34266,7 +34266,7 @@
       </c>
       <c r="G5" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week8.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week8.docx</t>
         </is>
       </c>
       <c r="H5" s="30" t="inlineStr">
@@ -34316,7 +34316,7 @@
       </c>
       <c r="G6" s="30" t="inlineStr">
         <is>
-          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/main/docs/Report/AI_Evidence/Week8.docx</t>
+          <t>https://github.com/vvtPhongdev/SE20A05Group7RMS/blob/docs/project-report-and-workflow-updates/docs/Report/AI_Evidence/Week8.docx</t>
         </is>
       </c>
       <c r="H6" s="30" t="inlineStr">

</xml_diff>